<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-17 03:22 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -6105,7 +6105,7 @@
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46184.1946494213</v>
+        <v>46190.12544563657</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>285</v>
@@ -6168,7 +6168,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46184.19464939815</v>
+        <v>46190.12544762732</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>290</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-22 17:16 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -5281,7 +5281,7 @@
       </c>
       <c r="C63" s="9"/>
       <c r="D63" s="8">
-        <v>46087.815567488426</v>
+        <v>46195.6882462963</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>240</v>
@@ -5326,9 +5326,11 @@
       <c r="B64" s="5">
         <v>46073.79484796296</v>
       </c>
-      <c r="C64" s="6"/>
+      <c r="C64" s="5">
+        <v>46195.68823886574</v>
+      </c>
       <c r="D64" s="5">
-        <v>46143.68356638889</v>
+        <v>46195.688256319445</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>243</v>
@@ -5376,10 +5378,10 @@
         <v>60</v>
       </c>
       <c r="T64" s="6">
-        <v>0</v>
-      </c>
-      <c r="U64" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U64" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5391,7 +5393,7 @@
       </c>
       <c r="C65" s="9"/>
       <c r="D65" s="8">
-        <v>46171.17405991898</v>
+        <v>46195.68826325232</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>246</v>
@@ -5441,8 +5443,8 @@
       <c r="T65" s="9">
         <v>0</v>
       </c>
-      <c r="U65" s="10" t="s">
-        <v>61</v>
+      <c r="U65" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5454,7 +5456,7 @@
       </c>
       <c r="C66" s="6"/>
       <c r="D66" s="5">
-        <v>46160.54837657408</v>
+        <v>46195.68826268519</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>250</v>
@@ -5504,8 +5506,8 @@
       <c r="T66" s="6">
         <v>0</v>
       </c>
-      <c r="U66" s="10" t="s">
-        <v>61</v>
+      <c r="U66" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5517,7 +5519,7 @@
       </c>
       <c r="C67" s="9"/>
       <c r="D67" s="8">
-        <v>46160.54616232638</v>
+        <v>46195.68826314815</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>253</v>
@@ -5567,8 +5569,8 @@
       <c r="T67" s="9">
         <v>0</v>
       </c>
-      <c r="U67" s="10" t="s">
-        <v>61</v>
+      <c r="U67" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5580,7 +5582,7 @@
       </c>
       <c r="C68" s="6"/>
       <c r="D68" s="5">
-        <v>46140.16812383102</v>
+        <v>46195.688253761575</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>256</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 13:19 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1003" uniqueCount="299">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="299">
   <si>
     <t>50001446-MINERA FRESNILLO</t>
   </si>
@@ -4415,7 +4415,7 @@
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46172.18038884259</v>
+        <v>46197.50927037037</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>189</v>
@@ -4463,8 +4463,8 @@
       <c r="T49" s="9">
         <v>0</v>
       </c>
-      <c r="U49" s="10" t="s">
-        <v>61</v>
+      <c r="U49" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -5279,9 +5279,11 @@
       <c r="B63" s="8">
         <v>46073.79484768519</v>
       </c>
-      <c r="C63" s="9"/>
+      <c r="C63" s="8">
+        <v>46197.50932107639</v>
+      </c>
       <c r="D63" s="8">
-        <v>46195.6882462963</v>
+        <v>46197.50933475695</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>240</v>
@@ -5316,8 +5318,12 @@
       <c r="Q63" s="9"/>
       <c r="R63" s="9"/>
       <c r="S63" s="9"/>
-      <c r="T63" s="9"/>
-      <c r="U63" s="9"/>
+      <c r="T63" s="9">
+        <v>1</v>
+      </c>
+      <c r="U63" s="11" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="64" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A64" s="4" t="s">
@@ -5391,9 +5397,11 @@
       <c r="B65" s="8">
         <v>46073.79484829861</v>
       </c>
-      <c r="C65" s="9"/>
+      <c r="C65" s="8">
+        <v>46197.50917609954</v>
+      </c>
       <c r="D65" s="8">
-        <v>46195.68826325232</v>
+        <v>46197.50919467593</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>246</v>
@@ -5441,10 +5449,10 @@
         <v>60</v>
       </c>
       <c r="T65" s="9">
-        <v>0</v>
-      </c>
-      <c r="U65" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U65" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5454,9 +5462,11 @@
       <c r="B66" s="5">
         <v>46073.79484857639</v>
       </c>
-      <c r="C66" s="6"/>
+      <c r="C66" s="5">
+        <v>46197.50918461806</v>
+      </c>
       <c r="D66" s="5">
-        <v>46195.68826268519</v>
+        <v>46197.50920605324</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>250</v>
@@ -5504,10 +5514,10 @@
         <v>60</v>
       </c>
       <c r="T66" s="6">
-        <v>0</v>
-      </c>
-      <c r="U66" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U66" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5517,9 +5527,11 @@
       <c r="B67" s="8">
         <v>46073.79484884259</v>
       </c>
-      <c r="C67" s="9"/>
+      <c r="C67" s="8">
+        <v>46197.50919322917</v>
+      </c>
       <c r="D67" s="8">
-        <v>46195.68826314815</v>
+        <v>46197.509207361116</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>253</v>
@@ -5567,10 +5579,10 @@
         <v>60</v>
       </c>
       <c r="T67" s="9">
-        <v>0</v>
-      </c>
-      <c r="U67" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U67" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5580,9 +5592,11 @@
       <c r="B68" s="5">
         <v>46076.6229305787</v>
       </c>
-      <c r="C68" s="6"/>
+      <c r="C68" s="5">
+        <v>46197.50920206019</v>
+      </c>
       <c r="D68" s="5">
-        <v>46195.688253761575</v>
+        <v>46197.50921739583</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>256</v>
@@ -5630,10 +5644,10 @@
         <v>60</v>
       </c>
       <c r="T68" s="6">
-        <v>0</v>
-      </c>
-      <c r="U68" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U68" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">
@@ -5643,9 +5657,11 @@
       <c r="B69" s="8">
         <v>46073.79484912037</v>
       </c>
-      <c r="C69" s="9"/>
+      <c r="C69" s="8">
+        <v>46197.5092531713</v>
+      </c>
       <c r="D69" s="8">
-        <v>46171.174060300924</v>
+        <v>46197.50926989583</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>192</v>
@@ -5691,10 +5707,10 @@
         <v>60</v>
       </c>
       <c r="T69" s="9">
-        <v>0</v>
-      </c>
-      <c r="U69" s="10" t="s">
-        <v>61</v>
+        <v>1</v>
+      </c>
+      <c r="U69" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="70" spans="1:21" x14ac:dyDescent="0.25">
@@ -5704,9 +5720,11 @@
       <c r="B70" s="5">
         <v>46073.794849432874</v>
       </c>
-      <c r="C70" s="6"/>
+      <c r="C70" s="5">
+        <v>46197.50929818287</v>
+      </c>
       <c r="D70" s="5">
-        <v>46173.191133125</v>
+        <v>46197.50932179399</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>193</v>
@@ -5752,10 +5770,10 @@
         <v>60</v>
       </c>
       <c r="T70" s="6">
-        <v>0</v>
-      </c>
-      <c r="U70" s="10" t="s">
-        <v>61</v>
+        <v>1</v>
+      </c>
+      <c r="U70" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">
@@ -5814,7 +5832,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46176.20449607639</v>
+        <v>46197.50931729167</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>267</v>
@@ -5862,8 +5880,8 @@
       <c r="T72" s="6">
         <v>0</v>
       </c>
-      <c r="U72" s="10" t="s">
-        <v>61</v>
+      <c r="U72" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 18:39 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -1626,13 +1626,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46073.79484634259</v>
+        <v>46073.62817967593</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.716893206016</v>
+        <v>46092.55022653935</v>
       </c>
       <c r="D4" s="5">
-        <v>46129.71434277778</v>
+        <v>46129.547676111106</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1675,13 +1675,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46073.794846689816</v>
+        <v>46073.62818002315</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.71686800926</v>
+        <v>46092.550201342594</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.877754201385</v>
+        <v>46133.71108753472</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1740,13 +1740,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46073.794847060184</v>
+        <v>46073.62818039352</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.716868564814</v>
+        <v>46092.55020189815</v>
       </c>
       <c r="D6" s="5">
-        <v>46134.64561201389</v>
+        <v>46134.47894534722</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1805,13 +1805,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46073.79484736111</v>
+        <v>46073.628180694446</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.71686905093</v>
+        <v>46092.55020238426</v>
       </c>
       <c r="D7" s="8">
-        <v>46134.64560787037</v>
+        <v>46134.478941203706</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1870,13 +1870,13 @@
         <v>41</v>
       </c>
       <c r="B8" s="5">
-        <v>46073.794847627316</v>
+        <v>46073.628180960644</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.71686943287</v>
+        <v>46092.5502027662</v>
       </c>
       <c r="D8" s="5">
-        <v>46134.64560351852</v>
+        <v>46134.478936851854</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>42</v>
@@ -1935,13 +1935,13 @@
         <v>45</v>
       </c>
       <c r="B9" s="8">
-        <v>46073.7948479051</v>
+        <v>46073.628181238426</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.71687001157</v>
+        <v>46092.55020334491</v>
       </c>
       <c r="D9" s="8">
-        <v>46134.64559775463</v>
+        <v>46134.478931087964</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>46</v>
@@ -2000,13 +2000,13 @@
         <v>48</v>
       </c>
       <c r="B10" s="5">
-        <v>46073.794848668986</v>
+        <v>46073.628182002314</v>
       </c>
       <c r="C10" s="5">
-        <v>46129.60128928241</v>
+        <v>46129.434622615736</v>
       </c>
       <c r="D10" s="5">
-        <v>46129.71438604167</v>
+        <v>46129.547719375</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>49</v>
@@ -2049,13 +2049,13 @@
         <v>51</v>
       </c>
       <c r="B11" s="8">
-        <v>46073.794848958336</v>
+        <v>46073.628182291664</v>
       </c>
       <c r="C11" s="8">
-        <v>46097.54943753472</v>
+        <v>46097.382770868055</v>
       </c>
       <c r="D11" s="8">
-        <v>46097.549452499996</v>
+        <v>46097.38278583333</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>52</v>
@@ -2114,13 +2114,13 @@
         <v>56</v>
       </c>
       <c r="B12" s="5">
-        <v>46073.79484923611</v>
+        <v>46073.628182569446</v>
       </c>
       <c r="C12" s="5">
-        <v>46129.60127643518</v>
+        <v>46129.43460976852</v>
       </c>
       <c r="D12" s="5">
-        <v>46154.171658692125</v>
+        <v>46154.00499202547</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -2179,13 +2179,13 @@
         <v>62</v>
       </c>
       <c r="B13" s="8">
-        <v>46073.794849513884</v>
+        <v>46073.62818284723</v>
       </c>
       <c r="C13" s="8">
-        <v>46097.54717446759</v>
+        <v>46097.380507800925</v>
       </c>
       <c r="D13" s="8">
-        <v>46129.71444074074</v>
+        <v>46129.547774074075</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>63</v>
@@ -2228,13 +2228,13 @@
         <v>65</v>
       </c>
       <c r="B14" s="5">
-        <v>46073.79484703703</v>
+        <v>46073.628180370375</v>
       </c>
       <c r="C14" s="5">
-        <v>46097.54673729167</v>
+        <v>46097.380070625004</v>
       </c>
       <c r="D14" s="5">
-        <v>46104.554936064815</v>
+        <v>46104.38826939814</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>66</v>
@@ -2293,13 +2293,13 @@
         <v>69</v>
       </c>
       <c r="B15" s="8">
-        <v>46073.794847592595</v>
+        <v>46073.62818092592</v>
       </c>
       <c r="C15" s="8">
-        <v>46097.54711586806</v>
+        <v>46097.38044920139</v>
       </c>
       <c r="D15" s="8">
-        <v>46104.55553096065</v>
+        <v>46104.388864293986</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>70</v>
@@ -2358,13 +2358,13 @@
         <v>73</v>
       </c>
       <c r="B16" s="5">
-        <v>46073.79484783565</v>
+        <v>46073.628181168984</v>
       </c>
       <c r="C16" s="5">
-        <v>46097.54692731482</v>
+        <v>46097.38026064815</v>
       </c>
       <c r="D16" s="5">
-        <v>46104.56897644676</v>
+        <v>46104.4023097801</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>74</v>
@@ -2423,13 +2423,13 @@
         <v>77</v>
       </c>
       <c r="B17" s="8">
-        <v>46073.79484809028</v>
+        <v>46073.62818142361</v>
       </c>
       <c r="C17" s="8">
-        <v>46097.5471527662</v>
+        <v>46097.38048609954</v>
       </c>
       <c r="D17" s="8">
-        <v>46100.77890356482</v>
+        <v>46100.612236898145</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>78</v>
@@ -2488,13 +2488,13 @@
         <v>82</v>
       </c>
       <c r="B18" s="5">
-        <v>46073.79484833333</v>
+        <v>46073.62818166667</v>
       </c>
       <c r="C18" s="5">
-        <v>46114.50368701389</v>
+        <v>46114.33702034722</v>
       </c>
       <c r="D18" s="5">
-        <v>46114.50370078704</v>
+        <v>46114.33703412037</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>83</v>
@@ -2541,13 +2541,13 @@
         <v>85</v>
       </c>
       <c r="B19" s="8">
-        <v>46073.79484857639</v>
+        <v>46073.62818190972</v>
       </c>
       <c r="C19" s="8">
-        <v>46101.81311775463</v>
+        <v>46101.64645108796</v>
       </c>
       <c r="D19" s="8">
-        <v>46104.56950603009</v>
+        <v>46104.40283936342</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>86</v>
@@ -2606,13 +2606,13 @@
         <v>89</v>
       </c>
       <c r="B20" s="5">
-        <v>46073.79484880787</v>
+        <v>46073.628182141205</v>
       </c>
       <c r="C20" s="5">
-        <v>46097.547598136574</v>
+        <v>46097.3809314699</v>
       </c>
       <c r="D20" s="5">
-        <v>46104.56972186343</v>
+        <v>46104.40305519676</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>90</v>
@@ -2671,13 +2671,13 @@
         <v>93</v>
       </c>
       <c r="B21" s="8">
-        <v>46073.79484905093</v>
+        <v>46073.62818238426</v>
       </c>
       <c r="C21" s="8">
-        <v>46097.54952784722</v>
+        <v>46097.38286118055</v>
       </c>
       <c r="D21" s="8">
-        <v>46104.570394375</v>
+        <v>46104.40372770833</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>94</v>
@@ -2736,13 +2736,13 @@
         <v>97</v>
       </c>
       <c r="B22" s="5">
-        <v>46073.79484929398</v>
+        <v>46073.62818262732</v>
       </c>
       <c r="C22" s="5">
-        <v>46101.81417637732</v>
+        <v>46101.647509710645</v>
       </c>
       <c r="D22" s="5">
-        <v>46101.814193136575</v>
+        <v>46101.64752646991</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>98</v>
@@ -2801,13 +2801,13 @@
         <v>101</v>
       </c>
       <c r="B23" s="8">
-        <v>46076.58214225694</v>
+        <v>46076.41547559028</v>
       </c>
       <c r="C23" s="8">
-        <v>46114.50366746528</v>
+        <v>46114.33700079861</v>
       </c>
       <c r="D23" s="8">
-        <v>46114.503793055555</v>
+        <v>46114.337126388884</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>102</v>
@@ -2866,13 +2866,13 @@
         <v>104</v>
       </c>
       <c r="B24" s="5">
-        <v>46073.79484642361</v>
+        <v>46073.62817975694</v>
       </c>
       <c r="C24" s="5">
-        <v>46097.54785292824</v>
+        <v>46097.38118626157</v>
       </c>
       <c r="D24" s="5">
-        <v>46100.778066307874</v>
+        <v>46100.6113996412</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>105</v>
@@ -2931,13 +2931,13 @@
         <v>109</v>
       </c>
       <c r="B25" s="8">
-        <v>46073.79484674768</v>
+        <v>46073.62818008102</v>
       </c>
       <c r="C25" s="8">
-        <v>46129.71470650463</v>
+        <v>46129.54803983796</v>
       </c>
       <c r="D25" s="8">
-        <v>46129.71472099537</v>
+        <v>46129.548054328705</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>110</v>
@@ -2984,13 +2984,13 @@
         <v>112</v>
       </c>
       <c r="B26" s="5">
-        <v>46073.79484700231</v>
+        <v>46073.62818033565</v>
       </c>
       <c r="C26" s="5">
-        <v>46097.54735603009</v>
+        <v>46097.380689363425</v>
       </c>
       <c r="D26" s="5">
-        <v>46134.20558688657</v>
+        <v>46134.03892021991</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>113</v>
@@ -3049,13 +3049,13 @@
         <v>117</v>
       </c>
       <c r="B27" s="8">
-        <v>46073.794847268524</v>
+        <v>46073.62818060185</v>
       </c>
       <c r="C27" s="8">
-        <v>46097.54729899306</v>
+        <v>46097.380632326385</v>
       </c>
       <c r="D27" s="8">
-        <v>46101.813124513894</v>
+        <v>46101.64645784722</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>118</v>
@@ -3114,13 +3114,13 @@
         <v>120</v>
       </c>
       <c r="B28" s="5">
-        <v>46073.79484752315</v>
+        <v>46073.62818085648</v>
       </c>
       <c r="C28" s="5">
-        <v>46097.54733972222</v>
+        <v>46097.38067305555</v>
       </c>
       <c r="D28" s="5">
-        <v>46097.54734099537</v>
+        <v>46097.3806743287</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>121</v>
@@ -3179,13 +3179,13 @@
         <v>123</v>
       </c>
       <c r="B29" s="8">
-        <v>46073.7948477662</v>
+        <v>46073.62818109954</v>
       </c>
       <c r="C29" s="8">
-        <v>46104.58757038195</v>
+        <v>46104.420903715276</v>
       </c>
       <c r="D29" s="8">
-        <v>46134.20558681713</v>
+        <v>46134.03892015046</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>124</v>
@@ -3244,13 +3244,13 @@
         <v>126</v>
       </c>
       <c r="B30" s="5">
-        <v>46073.79484803241</v>
+        <v>46073.62818136574</v>
       </c>
       <c r="C30" s="5">
-        <v>46104.58750148148</v>
+        <v>46104.42083481481</v>
       </c>
       <c r="D30" s="5">
-        <v>46104.58750311343</v>
+        <v>46104.42083644676</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>127</v>
@@ -3305,13 +3305,13 @@
         <v>129</v>
       </c>
       <c r="B31" s="8">
-        <v>46073.79484828704</v>
+        <v>46073.62818162037</v>
       </c>
       <c r="C31" s="8">
-        <v>46104.58755459491</v>
+        <v>46104.42088792824</v>
       </c>
       <c r="D31" s="8">
-        <v>46104.58755618056</v>
+        <v>46104.42088951389</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>130</v>
@@ -3366,13 +3366,13 @@
         <v>132</v>
       </c>
       <c r="B32" s="5">
-        <v>46073.79484853009</v>
+        <v>46073.62818186343</v>
       </c>
       <c r="C32" s="5">
-        <v>46104.583659386575</v>
+        <v>46104.41699271991</v>
       </c>
       <c r="D32" s="5">
-        <v>46104.58367331019</v>
+        <v>46104.41700664352</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>133</v>
@@ -3431,13 +3431,13 @@
         <v>135</v>
       </c>
       <c r="B33" s="8">
-        <v>46073.79484878472</v>
+        <v>46073.62818211806</v>
       </c>
       <c r="C33" s="8">
-        <v>46104.58357604167</v>
+        <v>46104.416909374995</v>
       </c>
       <c r="D33" s="8">
-        <v>46104.583577881946</v>
+        <v>46104.416911215274</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>136</v>
@@ -3492,13 +3492,13 @@
         <v>138</v>
       </c>
       <c r="B34" s="5">
-        <v>46073.79484700231</v>
+        <v>46073.62818033565</v>
       </c>
       <c r="C34" s="5">
-        <v>46104.58364541667</v>
+        <v>46104.41697875</v>
       </c>
       <c r="D34" s="5">
-        <v>46104.58364686342</v>
+        <v>46104.41698019676</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>139</v>
@@ -3553,13 +3553,13 @@
         <v>141</v>
       </c>
       <c r="B35" s="8">
-        <v>46073.79484739584</v>
+        <v>46073.62818072917</v>
       </c>
       <c r="C35" s="8">
-        <v>46104.584286990736</v>
+        <v>46104.41762032408</v>
       </c>
       <c r="D35" s="8">
-        <v>46165.2060525</v>
+        <v>46165.039385833334</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>142</v>
@@ -3618,13 +3618,13 @@
         <v>144</v>
       </c>
       <c r="B36" s="5">
-        <v>46073.79484769676</v>
+        <v>46073.62818103009</v>
       </c>
       <c r="C36" s="5">
-        <v>46104.58417509259</v>
+        <v>46104.417508425926</v>
       </c>
       <c r="D36" s="5">
-        <v>46104.58417674768</v>
+        <v>46104.41751008102</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>145</v>
@@ -3679,13 +3679,13 @@
         <v>147</v>
       </c>
       <c r="B37" s="8">
-        <v>46073.79484798611</v>
+        <v>46073.628181319444</v>
       </c>
       <c r="C37" s="8">
-        <v>46104.58422200232</v>
+        <v>46104.41755533565</v>
       </c>
       <c r="D37" s="8">
-        <v>46104.58422371528</v>
+        <v>46104.41755704861</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>148</v>
@@ -3740,13 +3740,13 @@
         <v>150</v>
       </c>
       <c r="B38" s="5">
-        <v>46073.79484826389</v>
+        <v>46073.62818159722</v>
       </c>
       <c r="C38" s="5">
-        <v>46104.58427152778</v>
+        <v>46104.41760486111</v>
       </c>
       <c r="D38" s="5">
-        <v>46104.58427320602</v>
+        <v>46104.417606539355</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>151</v>
@@ -3801,13 +3801,13 @@
         <v>153</v>
       </c>
       <c r="B39" s="8">
-        <v>46073.794848564816</v>
+        <v>46073.62818189815</v>
       </c>
       <c r="C39" s="8">
-        <v>46114.801113587964</v>
+        <v>46114.63444692129</v>
       </c>
       <c r="D39" s="8">
-        <v>46114.801124247686</v>
+        <v>46114.63445758102</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>154</v>
@@ -3866,13 +3866,13 @@
         <v>158</v>
       </c>
       <c r="B40" s="5">
-        <v>46073.79484883102</v>
+        <v>46073.62818216435</v>
       </c>
       <c r="C40" s="5">
-        <v>46112.591430416665</v>
+        <v>46112.42476375</v>
       </c>
       <c r="D40" s="5">
-        <v>46112.59143256945</v>
+        <v>46112.424765902775</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>159</v>
@@ -3927,13 +3927,13 @@
         <v>161</v>
       </c>
       <c r="B41" s="8">
-        <v>46073.79484913194</v>
+        <v>46073.628182465276</v>
       </c>
       <c r="C41" s="8">
-        <v>46114.80109980324</v>
+        <v>46114.63443313657</v>
       </c>
       <c r="D41" s="8">
-        <v>46114.80110109954</v>
+        <v>46114.63443443287</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>162</v>
@@ -3988,13 +3988,13 @@
         <v>164</v>
       </c>
       <c r="B42" s="5">
-        <v>46076.58266418982</v>
+        <v>46076.415997523145</v>
       </c>
       <c r="C42" s="5">
-        <v>46112.49794984954</v>
+        <v>46112.331283182866</v>
       </c>
       <c r="D42" s="5">
-        <v>46134.19208922454</v>
+        <v>46134.02542255787</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>165</v>
@@ -4053,13 +4053,13 @@
         <v>167</v>
       </c>
       <c r="B43" s="8">
-        <v>46076.58280495371</v>
+        <v>46076.41613828704</v>
       </c>
       <c r="C43" s="8">
-        <v>46129.7145863426</v>
+        <v>46129.547919675926</v>
       </c>
       <c r="D43" s="8">
-        <v>46129.714587407405</v>
+        <v>46129.54792074074</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>168</v>
@@ -4114,13 +4114,13 @@
         <v>170</v>
       </c>
       <c r="B44" s="5">
-        <v>46076.58302251158</v>
+        <v>46076.41635584491</v>
       </c>
       <c r="C44" s="5">
-        <v>46129.7146324537</v>
+        <v>46129.54796578704</v>
       </c>
       <c r="D44" s="5">
-        <v>46129.714633553245</v>
+        <v>46129.547966886574</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>171</v>
@@ -4175,11 +4175,11 @@
         <v>173</v>
       </c>
       <c r="B45" s="8">
-        <v>46073.794849467595</v>
+        <v>46073.62818280092</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="8">
-        <v>46114.798811886576</v>
+        <v>46114.632145219904</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>174</v>
@@ -4224,13 +4224,13 @@
         <v>176</v>
       </c>
       <c r="B46" s="5">
-        <v>46073.79484973379</v>
+        <v>46073.62818306713</v>
       </c>
       <c r="C46" s="5">
-        <v>46114.79848856482</v>
+        <v>46114.63182189815</v>
       </c>
       <c r="D46" s="5">
-        <v>46197.70688251157</v>
+        <v>46197.54021584491</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>177</v>
@@ -4289,13 +4289,13 @@
         <v>181</v>
       </c>
       <c r="B47" s="8">
-        <v>46073.79484638889</v>
+        <v>46073.62817972222</v>
       </c>
       <c r="C47" s="8">
-        <v>46114.79872664352</v>
+        <v>46114.63205997685</v>
       </c>
       <c r="D47" s="8">
-        <v>46197.70691572917</v>
+        <v>46197.5402490625</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>182</v>
@@ -4354,13 +4354,13 @@
         <v>185</v>
       </c>
       <c r="B48" s="5">
-        <v>46087.80996193287</v>
+        <v>46087.6432952662</v>
       </c>
       <c r="C48" s="5">
-        <v>46114.798792835645</v>
+        <v>46114.63212616898</v>
       </c>
       <c r="D48" s="5">
-        <v>46114.798815428236</v>
+        <v>46114.63214876158</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>186</v>
@@ -4417,11 +4417,11 @@
         <v>190</v>
       </c>
       <c r="B49" s="8">
-        <v>46087.810021701385</v>
+        <v>46087.64335503472</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46197.50927037037</v>
+        <v>46197.3426037037</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>191</v>
@@ -4478,13 +4478,13 @@
         <v>196</v>
       </c>
       <c r="B50" s="5">
-        <v>46073.79484671296</v>
+        <v>46073.6281800463</v>
       </c>
       <c r="C50" s="5">
-        <v>46121.673340787034</v>
+        <v>46121.50667412037</v>
       </c>
       <c r="D50" s="5">
-        <v>46121.67335355324</v>
+        <v>46121.50668688657</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>197</v>
@@ -4531,13 +4531,13 @@
         <v>199</v>
       </c>
       <c r="B51" s="8">
-        <v>46073.79484696759</v>
+        <v>46073.628180300926</v>
       </c>
       <c r="C51" s="8">
-        <v>46120.799450266204</v>
+        <v>46120.63278359953</v>
       </c>
       <c r="D51" s="8">
-        <v>46120.79946753472</v>
+        <v>46120.63280086806</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>200</v>
@@ -4596,13 +4596,13 @@
         <v>204</v>
       </c>
       <c r="B52" s="5">
-        <v>46073.794847233796</v>
+        <v>46073.62818056713</v>
       </c>
       <c r="C52" s="5">
-        <v>46121.67332476852</v>
+        <v>46121.50665810185</v>
       </c>
       <c r="D52" s="5">
-        <v>46121.67355936342</v>
+        <v>46121.50689269676</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>205</v>
@@ -4661,13 +4661,13 @@
         <v>209</v>
       </c>
       <c r="B53" s="8">
-        <v>46073.794847488425</v>
+        <v>46073.62818082176</v>
       </c>
       <c r="C53" s="8">
-        <v>46132.76737151621</v>
+        <v>46132.60070484954</v>
       </c>
       <c r="D53" s="8">
-        <v>46132.76738453704</v>
+        <v>46132.60071787037</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>210</v>
@@ -4714,13 +4714,13 @@
         <v>212</v>
       </c>
       <c r="B54" s="5">
-        <v>46073.79484775463</v>
+        <v>46073.62818108796</v>
       </c>
       <c r="C54" s="5">
-        <v>46120.79905210648</v>
+        <v>46120.632385439814</v>
       </c>
       <c r="D54" s="5">
-        <v>46132.92421190972</v>
+        <v>46132.757545243054</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>213</v>
@@ -4779,13 +4779,13 @@
         <v>217</v>
       </c>
       <c r="B55" s="8">
-        <v>46073.79484800926</v>
+        <v>46073.62818134259</v>
       </c>
       <c r="C55" s="8">
-        <v>46132.561391932875</v>
+        <v>46132.394725266204</v>
       </c>
       <c r="D55" s="8">
-        <v>46132.561408657406</v>
+        <v>46132.39474199074</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>218</v>
@@ -4844,13 +4844,13 @@
         <v>221</v>
       </c>
       <c r="B56" s="5">
-        <v>46073.79484829861</v>
+        <v>46073.628181631946</v>
       </c>
       <c r="C56" s="5">
-        <v>46132.76735306713</v>
+        <v>46132.60068640046</v>
       </c>
       <c r="D56" s="5">
-        <v>46132.76737177084</v>
+        <v>46132.60070510417</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>222</v>
@@ -4909,13 +4909,13 @@
         <v>225</v>
       </c>
       <c r="B57" s="8">
-        <v>46073.79484855324</v>
+        <v>46073.628181886575</v>
       </c>
       <c r="C57" s="8">
-        <v>46129.71626407407</v>
+        <v>46129.54959740741</v>
       </c>
       <c r="D57" s="8">
-        <v>46129.71634960648</v>
+        <v>46129.54968293982</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>197</v>
@@ -4958,13 +4958,13 @@
         <v>227</v>
       </c>
       <c r="B58" s="5">
-        <v>46073.79484880787</v>
+        <v>46073.628182141205</v>
       </c>
       <c r="C58" s="5">
-        <v>46122.61763545139</v>
+        <v>46122.450968784724</v>
       </c>
       <c r="D58" s="5">
-        <v>46122.61765378472</v>
+        <v>46122.450987118056</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>228</v>
@@ -5023,13 +5023,13 @@
         <v>230</v>
       </c>
       <c r="B59" s="8">
-        <v>46073.79484665509</v>
+        <v>46073.62817998843</v>
       </c>
       <c r="C59" s="8">
-        <v>46122.659079606485</v>
+        <v>46122.49241293981</v>
       </c>
       <c r="D59" s="8">
-        <v>46147.17597939815</v>
+        <v>46147.00931273148</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>58</v>
@@ -5088,13 +5088,13 @@
         <v>232</v>
       </c>
       <c r="B60" s="5">
-        <v>46073.794847129626</v>
+        <v>46073.62818046296</v>
       </c>
       <c r="C60" s="5">
-        <v>46127.669174490744</v>
+        <v>46127.50250782407</v>
       </c>
       <c r="D60" s="5">
-        <v>46147.17597951389</v>
+        <v>46147.00931284722</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>233</v>
@@ -5153,13 +5153,13 @@
         <v>235</v>
       </c>
       <c r="B61" s="8">
-        <v>46073.794847418976</v>
+        <v>46073.62818075232</v>
       </c>
       <c r="C61" s="8">
-        <v>46127.66922835648</v>
+        <v>46127.50256168982</v>
       </c>
       <c r="D61" s="8">
-        <v>46169.174760891205</v>
+        <v>46169.00809422454</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>236</v>
@@ -5218,13 +5218,13 @@
         <v>238</v>
       </c>
       <c r="B62" s="5">
-        <v>46076.583608553236</v>
+        <v>46076.41694188658</v>
       </c>
       <c r="C62" s="5">
-        <v>46129.7162494213</v>
+        <v>46129.549582754626</v>
       </c>
       <c r="D62" s="5">
-        <v>46136.200935636574</v>
+        <v>46136.0342689699</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>239</v>
@@ -5283,13 +5283,13 @@
         <v>241</v>
       </c>
       <c r="B63" s="8">
-        <v>46073.79484768519</v>
+        <v>46073.62818101852</v>
       </c>
       <c r="C63" s="8">
-        <v>46197.50932107639</v>
+        <v>46197.342654409724</v>
       </c>
       <c r="D63" s="8">
-        <v>46197.50933475695</v>
+        <v>46197.34266809028</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>242</v>
@@ -5336,13 +5336,13 @@
         <v>244</v>
       </c>
       <c r="B64" s="5">
-        <v>46073.79484796296</v>
+        <v>46073.6281812963</v>
       </c>
       <c r="C64" s="5">
-        <v>46195.68823886574</v>
+        <v>46195.521572199075</v>
       </c>
       <c r="D64" s="5">
-        <v>46195.688256319445</v>
+        <v>46195.52158965278</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>245</v>
@@ -5401,13 +5401,13 @@
         <v>247</v>
       </c>
       <c r="B65" s="8">
-        <v>46073.79484829861</v>
+        <v>46073.628181631946</v>
       </c>
       <c r="C65" s="8">
-        <v>46197.50917609954</v>
+        <v>46197.34250943287</v>
       </c>
       <c r="D65" s="8">
-        <v>46197.50919467593</v>
+        <v>46197.34252800926</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>248</v>
@@ -5466,13 +5466,13 @@
         <v>251</v>
       </c>
       <c r="B66" s="5">
-        <v>46073.79484857639</v>
+        <v>46073.62818190972</v>
       </c>
       <c r="C66" s="5">
-        <v>46197.50918461806</v>
+        <v>46197.34251795139</v>
       </c>
       <c r="D66" s="5">
-        <v>46197.50920605324</v>
+        <v>46197.34253938658</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>252</v>
@@ -5531,13 +5531,13 @@
         <v>254</v>
       </c>
       <c r="B67" s="8">
-        <v>46073.79484884259</v>
+        <v>46073.628182175926</v>
       </c>
       <c r="C67" s="8">
-        <v>46197.50919322917</v>
+        <v>46197.3425265625</v>
       </c>
       <c r="D67" s="8">
-        <v>46197.509207361116</v>
+        <v>46197.342540694444</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>255</v>
@@ -5596,13 +5596,13 @@
         <v>257</v>
       </c>
       <c r="B68" s="5">
-        <v>46076.6229305787</v>
+        <v>46076.45626391204</v>
       </c>
       <c r="C68" s="5">
-        <v>46197.50920206019</v>
+        <v>46197.342535393516</v>
       </c>
       <c r="D68" s="5">
-        <v>46197.50921739583</v>
+        <v>46197.34255072917</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>258</v>
@@ -5661,13 +5661,13 @@
         <v>260</v>
       </c>
       <c r="B69" s="8">
-        <v>46073.79484912037</v>
+        <v>46073.6281824537</v>
       </c>
       <c r="C69" s="8">
-        <v>46197.5092531713</v>
+        <v>46197.34258650463</v>
       </c>
       <c r="D69" s="8">
-        <v>46197.50926989583</v>
+        <v>46197.34260322917</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>194</v>
@@ -5724,13 +5724,13 @@
         <v>263</v>
       </c>
       <c r="B70" s="5">
-        <v>46073.794849432874</v>
+        <v>46073.6281827662</v>
       </c>
       <c r="C70" s="5">
-        <v>46197.50929818287</v>
+        <v>46197.34263151621</v>
       </c>
       <c r="D70" s="5">
-        <v>46197.50932179399</v>
+        <v>46197.342655127315</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>195</v>
@@ -5787,11 +5787,11 @@
         <v>265</v>
       </c>
       <c r="B71" s="8">
-        <v>46073.794846979166</v>
+        <v>46073.6281803125</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46090.66949746528</v>
+        <v>46090.50283079861</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>266</v>
@@ -5834,11 +5834,11 @@
         <v>268</v>
       </c>
       <c r="B72" s="5">
-        <v>46073.794847384255</v>
+        <v>46073.62818071759</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46197.50931729167</v>
+        <v>46197.342650624996</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>269</v>
@@ -5895,11 +5895,11 @@
         <v>273</v>
       </c>
       <c r="B73" s="8">
-        <v>46073.79484767361</v>
+        <v>46073.62818100695</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46179.16820392361</v>
+        <v>46179.00153725695</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>274</v>
@@ -5958,11 +5958,11 @@
         <v>277</v>
       </c>
       <c r="B74" s="5">
-        <v>46073.79484796296</v>
+        <v>46073.6281812963</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46182.18235991898</v>
+        <v>46182.01569325231</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>278</v>
@@ -6019,11 +6019,11 @@
         <v>280</v>
       </c>
       <c r="B75" s="8">
-        <v>46073.79484825231</v>
+        <v>46073.62818158565</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46183.188021875</v>
+        <v>46183.02135520833</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>281</v>
@@ -6080,11 +6080,11 @@
         <v>283</v>
       </c>
       <c r="B76" s="5">
-        <v>46073.79484855324</v>
+        <v>46073.628181886575</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46090.66953237269</v>
+        <v>46090.50286570602</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>284</v>
@@ -6127,11 +6127,11 @@
         <v>286</v>
       </c>
       <c r="B77" s="8">
-        <v>46073.79484886574</v>
+        <v>46073.62818219907</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46192.175525451385</v>
+        <v>46192.00885878473</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>287</v>
@@ -6190,11 +6190,11 @@
         <v>291</v>
       </c>
       <c r="B78" s="5">
-        <v>46073.79484915509</v>
+        <v>46073.62818248842</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46192.175525451385</v>
+        <v>46192.00885878473</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>292</v>
@@ -6253,11 +6253,11 @@
         <v>293</v>
       </c>
       <c r="B79" s="8">
-        <v>46090.64638520833</v>
+        <v>46090.47971854167</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46090.66956530092</v>
+        <v>46090.50289863426</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>294</v>
@@ -6300,11 +6300,11 @@
         <v>296</v>
       </c>
       <c r="B80" s="5">
-        <v>46090.646490810184</v>
+        <v>46090.47982414352</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46191.18765634259</v>
+        <v>46191.020989675926</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>297</v>
@@ -6363,11 +6363,11 @@
         <v>299</v>
       </c>
       <c r="B81" s="8">
-        <v>46090.64689480324</v>
+        <v>46090.48022813657</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46192.17605807871</v>
+        <v>46192.00939141204</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>300</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 19:07 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -1626,13 +1626,13 @@
         <v>23</v>
       </c>
       <c r="B4" s="5">
-        <v>46073.62817967593</v>
+        <v>46073.79484634259</v>
       </c>
       <c r="C4" s="5">
-        <v>46092.55022653935</v>
+        <v>46092.716893206016</v>
       </c>
       <c r="D4" s="5">
-        <v>46129.547676111106</v>
+        <v>46129.71434277778</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1675,13 +1675,13 @@
         <v>27</v>
       </c>
       <c r="B5" s="8">
-        <v>46073.62818002315</v>
+        <v>46073.794846689816</v>
       </c>
       <c r="C5" s="8">
-        <v>46092.550201342594</v>
+        <v>46092.71686800926</v>
       </c>
       <c r="D5" s="8">
-        <v>46133.71108753472</v>
+        <v>46133.877754201385</v>
       </c>
       <c r="E5" s="9" t="s">
         <v>28</v>
@@ -1740,13 +1740,13 @@
         <v>34</v>
       </c>
       <c r="B6" s="5">
-        <v>46073.62818039352</v>
+        <v>46073.794847060184</v>
       </c>
       <c r="C6" s="5">
-        <v>46092.55020189815</v>
+        <v>46092.716868564814</v>
       </c>
       <c r="D6" s="5">
-        <v>46134.47894534722</v>
+        <v>46134.64561201389</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>35</v>
@@ -1805,13 +1805,13 @@
         <v>38</v>
       </c>
       <c r="B7" s="8">
-        <v>46073.628180694446</v>
+        <v>46073.79484736111</v>
       </c>
       <c r="C7" s="8">
-        <v>46092.55020238426</v>
+        <v>46092.71686905093</v>
       </c>
       <c r="D7" s="8">
-        <v>46134.478941203706</v>
+        <v>46134.64560787037</v>
       </c>
       <c r="E7" s="9" t="s">
         <v>39</v>
@@ -1870,13 +1870,13 @@
         <v>41</v>
       </c>
       <c r="B8" s="5">
-        <v>46073.628180960644</v>
+        <v>46073.794847627316</v>
       </c>
       <c r="C8" s="5">
-        <v>46092.5502027662</v>
+        <v>46092.71686943287</v>
       </c>
       <c r="D8" s="5">
-        <v>46134.478936851854</v>
+        <v>46134.64560351852</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>42</v>
@@ -1935,13 +1935,13 @@
         <v>45</v>
       </c>
       <c r="B9" s="8">
-        <v>46073.628181238426</v>
+        <v>46073.7948479051</v>
       </c>
       <c r="C9" s="8">
-        <v>46092.55020334491</v>
+        <v>46092.71687001157</v>
       </c>
       <c r="D9" s="8">
-        <v>46134.478931087964</v>
+        <v>46134.64559775463</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>46</v>
@@ -2000,13 +2000,13 @@
         <v>48</v>
       </c>
       <c r="B10" s="5">
-        <v>46073.628182002314</v>
+        <v>46073.794848668986</v>
       </c>
       <c r="C10" s="5">
-        <v>46129.434622615736</v>
+        <v>46129.60128928241</v>
       </c>
       <c r="D10" s="5">
-        <v>46129.547719375</v>
+        <v>46129.71438604167</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>49</v>
@@ -2049,13 +2049,13 @@
         <v>51</v>
       </c>
       <c r="B11" s="8">
-        <v>46073.628182291664</v>
+        <v>46073.794848958336</v>
       </c>
       <c r="C11" s="8">
-        <v>46097.382770868055</v>
+        <v>46097.54943753472</v>
       </c>
       <c r="D11" s="8">
-        <v>46097.38278583333</v>
+        <v>46097.549452499996</v>
       </c>
       <c r="E11" s="9" t="s">
         <v>52</v>
@@ -2114,13 +2114,13 @@
         <v>56</v>
       </c>
       <c r="B12" s="5">
-        <v>46073.628182569446</v>
+        <v>46073.79484923611</v>
       </c>
       <c r="C12" s="5">
-        <v>46129.43460976852</v>
+        <v>46129.60127643518</v>
       </c>
       <c r="D12" s="5">
-        <v>46154.00499202547</v>
+        <v>46154.171658692125</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -2179,13 +2179,13 @@
         <v>62</v>
       </c>
       <c r="B13" s="8">
-        <v>46073.62818284723</v>
+        <v>46073.794849513884</v>
       </c>
       <c r="C13" s="8">
-        <v>46097.380507800925</v>
+        <v>46097.54717446759</v>
       </c>
       <c r="D13" s="8">
-        <v>46129.547774074075</v>
+        <v>46129.71444074074</v>
       </c>
       <c r="E13" s="9" t="s">
         <v>63</v>
@@ -2228,13 +2228,13 @@
         <v>65</v>
       </c>
       <c r="B14" s="5">
-        <v>46073.628180370375</v>
+        <v>46073.79484703703</v>
       </c>
       <c r="C14" s="5">
-        <v>46097.380070625004</v>
+        <v>46097.54673729167</v>
       </c>
       <c r="D14" s="5">
-        <v>46104.38826939814</v>
+        <v>46104.554936064815</v>
       </c>
       <c r="E14" s="6" t="s">
         <v>66</v>
@@ -2293,13 +2293,13 @@
         <v>69</v>
       </c>
       <c r="B15" s="8">
-        <v>46073.62818092592</v>
+        <v>46073.794847592595</v>
       </c>
       <c r="C15" s="8">
-        <v>46097.38044920139</v>
+        <v>46097.54711586806</v>
       </c>
       <c r="D15" s="8">
-        <v>46104.388864293986</v>
+        <v>46104.55553096065</v>
       </c>
       <c r="E15" s="9" t="s">
         <v>70</v>
@@ -2358,13 +2358,13 @@
         <v>73</v>
       </c>
       <c r="B16" s="5">
-        <v>46073.628181168984</v>
+        <v>46073.79484783565</v>
       </c>
       <c r="C16" s="5">
-        <v>46097.38026064815</v>
+        <v>46097.54692731482</v>
       </c>
       <c r="D16" s="5">
-        <v>46104.4023097801</v>
+        <v>46104.56897644676</v>
       </c>
       <c r="E16" s="6" t="s">
         <v>74</v>
@@ -2423,13 +2423,13 @@
         <v>77</v>
       </c>
       <c r="B17" s="8">
-        <v>46073.62818142361</v>
+        <v>46073.79484809028</v>
       </c>
       <c r="C17" s="8">
-        <v>46097.38048609954</v>
+        <v>46097.5471527662</v>
       </c>
       <c r="D17" s="8">
-        <v>46100.612236898145</v>
+        <v>46100.77890356482</v>
       </c>
       <c r="E17" s="9" t="s">
         <v>78</v>
@@ -2488,13 +2488,13 @@
         <v>82</v>
       </c>
       <c r="B18" s="5">
-        <v>46073.62818166667</v>
+        <v>46073.79484833333</v>
       </c>
       <c r="C18" s="5">
-        <v>46114.33702034722</v>
+        <v>46114.50368701389</v>
       </c>
       <c r="D18" s="5">
-        <v>46114.33703412037</v>
+        <v>46114.50370078704</v>
       </c>
       <c r="E18" s="6" t="s">
         <v>83</v>
@@ -2541,13 +2541,13 @@
         <v>85</v>
       </c>
       <c r="B19" s="8">
-        <v>46073.62818190972</v>
+        <v>46073.79484857639</v>
       </c>
       <c r="C19" s="8">
-        <v>46101.64645108796</v>
+        <v>46101.81311775463</v>
       </c>
       <c r="D19" s="8">
-        <v>46104.40283936342</v>
+        <v>46104.56950603009</v>
       </c>
       <c r="E19" s="9" t="s">
         <v>86</v>
@@ -2606,13 +2606,13 @@
         <v>89</v>
       </c>
       <c r="B20" s="5">
-        <v>46073.628182141205</v>
+        <v>46073.79484880787</v>
       </c>
       <c r="C20" s="5">
-        <v>46097.3809314699</v>
+        <v>46097.547598136574</v>
       </c>
       <c r="D20" s="5">
-        <v>46104.40305519676</v>
+        <v>46104.56972186343</v>
       </c>
       <c r="E20" s="6" t="s">
         <v>90</v>
@@ -2671,13 +2671,13 @@
         <v>93</v>
       </c>
       <c r="B21" s="8">
-        <v>46073.62818238426</v>
+        <v>46073.79484905093</v>
       </c>
       <c r="C21" s="8">
-        <v>46097.38286118055</v>
+        <v>46097.54952784722</v>
       </c>
       <c r="D21" s="8">
-        <v>46104.40372770833</v>
+        <v>46104.570394375</v>
       </c>
       <c r="E21" s="9" t="s">
         <v>94</v>
@@ -2736,13 +2736,13 @@
         <v>97</v>
       </c>
       <c r="B22" s="5">
-        <v>46073.62818262732</v>
+        <v>46073.79484929398</v>
       </c>
       <c r="C22" s="5">
-        <v>46101.647509710645</v>
+        <v>46101.81417637732</v>
       </c>
       <c r="D22" s="5">
-        <v>46101.64752646991</v>
+        <v>46101.814193136575</v>
       </c>
       <c r="E22" s="6" t="s">
         <v>98</v>
@@ -2801,13 +2801,13 @@
         <v>101</v>
       </c>
       <c r="B23" s="8">
-        <v>46076.41547559028</v>
+        <v>46076.58214225694</v>
       </c>
       <c r="C23" s="8">
-        <v>46114.33700079861</v>
+        <v>46114.50366746528</v>
       </c>
       <c r="D23" s="8">
-        <v>46114.337126388884</v>
+        <v>46114.503793055555</v>
       </c>
       <c r="E23" s="9" t="s">
         <v>102</v>
@@ -2866,13 +2866,13 @@
         <v>104</v>
       </c>
       <c r="B24" s="5">
-        <v>46073.62817975694</v>
+        <v>46073.79484642361</v>
       </c>
       <c r="C24" s="5">
-        <v>46097.38118626157</v>
+        <v>46097.54785292824</v>
       </c>
       <c r="D24" s="5">
-        <v>46100.6113996412</v>
+        <v>46100.778066307874</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>105</v>
@@ -2931,13 +2931,13 @@
         <v>109</v>
       </c>
       <c r="B25" s="8">
-        <v>46073.62818008102</v>
+        <v>46073.79484674768</v>
       </c>
       <c r="C25" s="8">
-        <v>46129.54803983796</v>
+        <v>46129.71470650463</v>
       </c>
       <c r="D25" s="8">
-        <v>46129.548054328705</v>
+        <v>46129.71472099537</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>110</v>
@@ -2984,13 +2984,13 @@
         <v>112</v>
       </c>
       <c r="B26" s="5">
-        <v>46073.62818033565</v>
+        <v>46073.79484700231</v>
       </c>
       <c r="C26" s="5">
-        <v>46097.380689363425</v>
+        <v>46097.54735603009</v>
       </c>
       <c r="D26" s="5">
-        <v>46134.03892021991</v>
+        <v>46134.20558688657</v>
       </c>
       <c r="E26" s="6" t="s">
         <v>113</v>
@@ -3049,13 +3049,13 @@
         <v>117</v>
       </c>
       <c r="B27" s="8">
-        <v>46073.62818060185</v>
+        <v>46073.794847268524</v>
       </c>
       <c r="C27" s="8">
-        <v>46097.380632326385</v>
+        <v>46097.54729899306</v>
       </c>
       <c r="D27" s="8">
-        <v>46101.64645784722</v>
+        <v>46101.813124513894</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>118</v>
@@ -3114,13 +3114,13 @@
         <v>120</v>
       </c>
       <c r="B28" s="5">
-        <v>46073.62818085648</v>
+        <v>46073.79484752315</v>
       </c>
       <c r="C28" s="5">
-        <v>46097.38067305555</v>
+        <v>46097.54733972222</v>
       </c>
       <c r="D28" s="5">
-        <v>46097.3806743287</v>
+        <v>46097.54734099537</v>
       </c>
       <c r="E28" s="6" t="s">
         <v>121</v>
@@ -3179,13 +3179,13 @@
         <v>123</v>
       </c>
       <c r="B29" s="8">
-        <v>46073.62818109954</v>
+        <v>46073.7948477662</v>
       </c>
       <c r="C29" s="8">
-        <v>46104.420903715276</v>
+        <v>46104.58757038195</v>
       </c>
       <c r="D29" s="8">
-        <v>46134.03892015046</v>
+        <v>46134.20558681713</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>124</v>
@@ -3244,13 +3244,13 @@
         <v>126</v>
       </c>
       <c r="B30" s="5">
-        <v>46073.62818136574</v>
+        <v>46073.79484803241</v>
       </c>
       <c r="C30" s="5">
-        <v>46104.42083481481</v>
+        <v>46104.58750148148</v>
       </c>
       <c r="D30" s="5">
-        <v>46104.42083644676</v>
+        <v>46104.58750311343</v>
       </c>
       <c r="E30" s="6" t="s">
         <v>127</v>
@@ -3305,13 +3305,13 @@
         <v>129</v>
       </c>
       <c r="B31" s="8">
-        <v>46073.62818162037</v>
+        <v>46073.79484828704</v>
       </c>
       <c r="C31" s="8">
-        <v>46104.42088792824</v>
+        <v>46104.58755459491</v>
       </c>
       <c r="D31" s="8">
-        <v>46104.42088951389</v>
+        <v>46104.58755618056</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>130</v>
@@ -3366,13 +3366,13 @@
         <v>132</v>
       </c>
       <c r="B32" s="5">
-        <v>46073.62818186343</v>
+        <v>46073.79484853009</v>
       </c>
       <c r="C32" s="5">
-        <v>46104.41699271991</v>
+        <v>46104.583659386575</v>
       </c>
       <c r="D32" s="5">
-        <v>46104.41700664352</v>
+        <v>46104.58367331019</v>
       </c>
       <c r="E32" s="6" t="s">
         <v>133</v>
@@ -3431,13 +3431,13 @@
         <v>135</v>
       </c>
       <c r="B33" s="8">
-        <v>46073.62818211806</v>
+        <v>46073.79484878472</v>
       </c>
       <c r="C33" s="8">
-        <v>46104.416909374995</v>
+        <v>46104.58357604167</v>
       </c>
       <c r="D33" s="8">
-        <v>46104.416911215274</v>
+        <v>46104.583577881946</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>136</v>
@@ -3492,13 +3492,13 @@
         <v>138</v>
       </c>
       <c r="B34" s="5">
-        <v>46073.62818033565</v>
+        <v>46073.79484700231</v>
       </c>
       <c r="C34" s="5">
-        <v>46104.41697875</v>
+        <v>46104.58364541667</v>
       </c>
       <c r="D34" s="5">
-        <v>46104.41698019676</v>
+        <v>46104.58364686342</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>139</v>
@@ -3553,13 +3553,13 @@
         <v>141</v>
       </c>
       <c r="B35" s="8">
-        <v>46073.62818072917</v>
+        <v>46073.79484739584</v>
       </c>
       <c r="C35" s="8">
-        <v>46104.41762032408</v>
+        <v>46104.584286990736</v>
       </c>
       <c r="D35" s="8">
-        <v>46165.039385833334</v>
+        <v>46165.2060525</v>
       </c>
       <c r="E35" s="9" t="s">
         <v>142</v>
@@ -3618,13 +3618,13 @@
         <v>144</v>
       </c>
       <c r="B36" s="5">
-        <v>46073.62818103009</v>
+        <v>46073.79484769676</v>
       </c>
       <c r="C36" s="5">
-        <v>46104.417508425926</v>
+        <v>46104.58417509259</v>
       </c>
       <c r="D36" s="5">
-        <v>46104.41751008102</v>
+        <v>46104.58417674768</v>
       </c>
       <c r="E36" s="6" t="s">
         <v>145</v>
@@ -3679,13 +3679,13 @@
         <v>147</v>
       </c>
       <c r="B37" s="8">
-        <v>46073.628181319444</v>
+        <v>46073.79484798611</v>
       </c>
       <c r="C37" s="8">
-        <v>46104.41755533565</v>
+        <v>46104.58422200232</v>
       </c>
       <c r="D37" s="8">
-        <v>46104.41755704861</v>
+        <v>46104.58422371528</v>
       </c>
       <c r="E37" s="9" t="s">
         <v>148</v>
@@ -3740,13 +3740,13 @@
         <v>150</v>
       </c>
       <c r="B38" s="5">
-        <v>46073.62818159722</v>
+        <v>46073.79484826389</v>
       </c>
       <c r="C38" s="5">
-        <v>46104.41760486111</v>
+        <v>46104.58427152778</v>
       </c>
       <c r="D38" s="5">
-        <v>46104.417606539355</v>
+        <v>46104.58427320602</v>
       </c>
       <c r="E38" s="6" t="s">
         <v>151</v>
@@ -3801,13 +3801,13 @@
         <v>153</v>
       </c>
       <c r="B39" s="8">
-        <v>46073.62818189815</v>
+        <v>46073.794848564816</v>
       </c>
       <c r="C39" s="8">
-        <v>46114.63444692129</v>
+        <v>46114.801113587964</v>
       </c>
       <c r="D39" s="8">
-        <v>46114.63445758102</v>
+        <v>46114.801124247686</v>
       </c>
       <c r="E39" s="9" t="s">
         <v>154</v>
@@ -3866,13 +3866,13 @@
         <v>158</v>
       </c>
       <c r="B40" s="5">
-        <v>46073.62818216435</v>
+        <v>46073.79484883102</v>
       </c>
       <c r="C40" s="5">
-        <v>46112.42476375</v>
+        <v>46112.591430416665</v>
       </c>
       <c r="D40" s="5">
-        <v>46112.424765902775</v>
+        <v>46112.59143256945</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>159</v>
@@ -3927,13 +3927,13 @@
         <v>161</v>
       </c>
       <c r="B41" s="8">
-        <v>46073.628182465276</v>
+        <v>46073.79484913194</v>
       </c>
       <c r="C41" s="8">
-        <v>46114.63443313657</v>
+        <v>46114.80109980324</v>
       </c>
       <c r="D41" s="8">
-        <v>46114.63443443287</v>
+        <v>46114.80110109954</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>162</v>
@@ -3988,13 +3988,13 @@
         <v>164</v>
       </c>
       <c r="B42" s="5">
-        <v>46076.415997523145</v>
+        <v>46076.58266418982</v>
       </c>
       <c r="C42" s="5">
-        <v>46112.331283182866</v>
+        <v>46112.49794984954</v>
       </c>
       <c r="D42" s="5">
-        <v>46134.02542255787</v>
+        <v>46134.19208922454</v>
       </c>
       <c r="E42" s="6" t="s">
         <v>165</v>
@@ -4053,13 +4053,13 @@
         <v>167</v>
       </c>
       <c r="B43" s="8">
-        <v>46076.41613828704</v>
+        <v>46076.58280495371</v>
       </c>
       <c r="C43" s="8">
-        <v>46129.547919675926</v>
+        <v>46129.7145863426</v>
       </c>
       <c r="D43" s="8">
-        <v>46129.54792074074</v>
+        <v>46129.714587407405</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>168</v>
@@ -4114,13 +4114,13 @@
         <v>170</v>
       </c>
       <c r="B44" s="5">
-        <v>46076.41635584491</v>
+        <v>46076.58302251158</v>
       </c>
       <c r="C44" s="5">
-        <v>46129.54796578704</v>
+        <v>46129.7146324537</v>
       </c>
       <c r="D44" s="5">
-        <v>46129.547966886574</v>
+        <v>46129.714633553245</v>
       </c>
       <c r="E44" s="6" t="s">
         <v>171</v>
@@ -4175,11 +4175,11 @@
         <v>173</v>
       </c>
       <c r="B45" s="8">
-        <v>46073.62818280092</v>
+        <v>46073.794849467595</v>
       </c>
       <c r="C45" s="9"/>
       <c r="D45" s="8">
-        <v>46114.632145219904</v>
+        <v>46114.798811886576</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>174</v>
@@ -4224,13 +4224,13 @@
         <v>176</v>
       </c>
       <c r="B46" s="5">
-        <v>46073.62818306713</v>
+        <v>46073.79484973379</v>
       </c>
       <c r="C46" s="5">
-        <v>46114.63182189815</v>
+        <v>46114.79848856482</v>
       </c>
       <c r="D46" s="5">
-        <v>46197.54021584491</v>
+        <v>46197.70688251157</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>177</v>
@@ -4289,13 +4289,13 @@
         <v>181</v>
       </c>
       <c r="B47" s="8">
-        <v>46073.62817972222</v>
+        <v>46073.79484638889</v>
       </c>
       <c r="C47" s="8">
-        <v>46114.63205997685</v>
+        <v>46114.79872664352</v>
       </c>
       <c r="D47" s="8">
-        <v>46197.5402490625</v>
+        <v>46197.70691572917</v>
       </c>
       <c r="E47" s="9" t="s">
         <v>182</v>
@@ -4354,13 +4354,13 @@
         <v>185</v>
       </c>
       <c r="B48" s="5">
-        <v>46087.6432952662</v>
+        <v>46087.80996193287</v>
       </c>
       <c r="C48" s="5">
-        <v>46114.63212616898</v>
+        <v>46114.798792835645</v>
       </c>
       <c r="D48" s="5">
-        <v>46114.63214876158</v>
+        <v>46114.798815428236</v>
       </c>
       <c r="E48" s="6" t="s">
         <v>186</v>
@@ -4417,11 +4417,11 @@
         <v>190</v>
       </c>
       <c r="B49" s="8">
-        <v>46087.64335503472</v>
+        <v>46087.810021701385</v>
       </c>
       <c r="C49" s="9"/>
       <c r="D49" s="8">
-        <v>46197.3426037037</v>
+        <v>46197.50927037037</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>191</v>
@@ -4478,13 +4478,13 @@
         <v>196</v>
       </c>
       <c r="B50" s="5">
-        <v>46073.6281800463</v>
+        <v>46073.79484671296</v>
       </c>
       <c r="C50" s="5">
-        <v>46121.50667412037</v>
+        <v>46121.673340787034</v>
       </c>
       <c r="D50" s="5">
-        <v>46121.50668688657</v>
+        <v>46121.67335355324</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>197</v>
@@ -4531,13 +4531,13 @@
         <v>199</v>
       </c>
       <c r="B51" s="8">
-        <v>46073.628180300926</v>
+        <v>46073.79484696759</v>
       </c>
       <c r="C51" s="8">
-        <v>46120.63278359953</v>
+        <v>46120.799450266204</v>
       </c>
       <c r="D51" s="8">
-        <v>46120.63280086806</v>
+        <v>46120.79946753472</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>200</v>
@@ -4596,13 +4596,13 @@
         <v>204</v>
       </c>
       <c r="B52" s="5">
-        <v>46073.62818056713</v>
+        <v>46073.794847233796</v>
       </c>
       <c r="C52" s="5">
-        <v>46121.50665810185</v>
+        <v>46121.67332476852</v>
       </c>
       <c r="D52" s="5">
-        <v>46121.50689269676</v>
+        <v>46121.67355936342</v>
       </c>
       <c r="E52" s="6" t="s">
         <v>205</v>
@@ -4661,13 +4661,13 @@
         <v>209</v>
       </c>
       <c r="B53" s="8">
-        <v>46073.62818082176</v>
+        <v>46073.794847488425</v>
       </c>
       <c r="C53" s="8">
-        <v>46132.60070484954</v>
+        <v>46132.76737151621</v>
       </c>
       <c r="D53" s="8">
-        <v>46132.60071787037</v>
+        <v>46132.76738453704</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>210</v>
@@ -4714,13 +4714,13 @@
         <v>212</v>
       </c>
       <c r="B54" s="5">
-        <v>46073.62818108796</v>
+        <v>46073.79484775463</v>
       </c>
       <c r="C54" s="5">
-        <v>46120.632385439814</v>
+        <v>46120.79905210648</v>
       </c>
       <c r="D54" s="5">
-        <v>46132.757545243054</v>
+        <v>46132.92421190972</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>213</v>
@@ -4779,13 +4779,13 @@
         <v>217</v>
       </c>
       <c r="B55" s="8">
-        <v>46073.62818134259</v>
+        <v>46073.79484800926</v>
       </c>
       <c r="C55" s="8">
-        <v>46132.394725266204</v>
+        <v>46132.561391932875</v>
       </c>
       <c r="D55" s="8">
-        <v>46132.39474199074</v>
+        <v>46132.561408657406</v>
       </c>
       <c r="E55" s="9" t="s">
         <v>218</v>
@@ -4844,13 +4844,13 @@
         <v>221</v>
       </c>
       <c r="B56" s="5">
-        <v>46073.628181631946</v>
+        <v>46073.79484829861</v>
       </c>
       <c r="C56" s="5">
-        <v>46132.60068640046</v>
+        <v>46132.76735306713</v>
       </c>
       <c r="D56" s="5">
-        <v>46132.60070510417</v>
+        <v>46132.76737177084</v>
       </c>
       <c r="E56" s="6" t="s">
         <v>222</v>
@@ -4909,13 +4909,13 @@
         <v>225</v>
       </c>
       <c r="B57" s="8">
-        <v>46073.628181886575</v>
+        <v>46073.79484855324</v>
       </c>
       <c r="C57" s="8">
-        <v>46129.54959740741</v>
+        <v>46129.71626407407</v>
       </c>
       <c r="D57" s="8">
-        <v>46129.54968293982</v>
+        <v>46129.71634960648</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>197</v>
@@ -4958,13 +4958,13 @@
         <v>227</v>
       </c>
       <c r="B58" s="5">
-        <v>46073.628182141205</v>
+        <v>46073.79484880787</v>
       </c>
       <c r="C58" s="5">
-        <v>46122.450968784724</v>
+        <v>46122.61763545139</v>
       </c>
       <c r="D58" s="5">
-        <v>46122.450987118056</v>
+        <v>46122.61765378472</v>
       </c>
       <c r="E58" s="6" t="s">
         <v>228</v>
@@ -5023,13 +5023,13 @@
         <v>230</v>
       </c>
       <c r="B59" s="8">
-        <v>46073.62817998843</v>
+        <v>46073.79484665509</v>
       </c>
       <c r="C59" s="8">
-        <v>46122.49241293981</v>
+        <v>46122.659079606485</v>
       </c>
       <c r="D59" s="8">
-        <v>46147.00931273148</v>
+        <v>46147.17597939815</v>
       </c>
       <c r="E59" s="9" t="s">
         <v>58</v>
@@ -5088,13 +5088,13 @@
         <v>232</v>
       </c>
       <c r="B60" s="5">
-        <v>46073.62818046296</v>
+        <v>46073.794847129626</v>
       </c>
       <c r="C60" s="5">
-        <v>46127.50250782407</v>
+        <v>46127.669174490744</v>
       </c>
       <c r="D60" s="5">
-        <v>46147.00931284722</v>
+        <v>46147.17597951389</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>233</v>
@@ -5153,13 +5153,13 @@
         <v>235</v>
       </c>
       <c r="B61" s="8">
-        <v>46073.62818075232</v>
+        <v>46073.794847418976</v>
       </c>
       <c r="C61" s="8">
-        <v>46127.50256168982</v>
+        <v>46127.66922835648</v>
       </c>
       <c r="D61" s="8">
-        <v>46169.00809422454</v>
+        <v>46169.174760891205</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>236</v>
@@ -5218,13 +5218,13 @@
         <v>238</v>
       </c>
       <c r="B62" s="5">
-        <v>46076.41694188658</v>
+        <v>46076.583608553236</v>
       </c>
       <c r="C62" s="5">
-        <v>46129.549582754626</v>
+        <v>46129.7162494213</v>
       </c>
       <c r="D62" s="5">
-        <v>46136.0342689699</v>
+        <v>46136.200935636574</v>
       </c>
       <c r="E62" s="6" t="s">
         <v>239</v>
@@ -5283,13 +5283,13 @@
         <v>241</v>
       </c>
       <c r="B63" s="8">
-        <v>46073.62818101852</v>
+        <v>46073.79484768519</v>
       </c>
       <c r="C63" s="8">
-        <v>46197.342654409724</v>
+        <v>46197.50932107639</v>
       </c>
       <c r="D63" s="8">
-        <v>46197.34266809028</v>
+        <v>46197.50933475695</v>
       </c>
       <c r="E63" s="9" t="s">
         <v>242</v>
@@ -5336,13 +5336,13 @@
         <v>244</v>
       </c>
       <c r="B64" s="5">
-        <v>46073.6281812963</v>
+        <v>46073.79484796296</v>
       </c>
       <c r="C64" s="5">
-        <v>46195.521572199075</v>
+        <v>46195.68823886574</v>
       </c>
       <c r="D64" s="5">
-        <v>46195.52158965278</v>
+        <v>46195.688256319445</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>245</v>
@@ -5401,13 +5401,13 @@
         <v>247</v>
       </c>
       <c r="B65" s="8">
-        <v>46073.628181631946</v>
+        <v>46073.79484829861</v>
       </c>
       <c r="C65" s="8">
-        <v>46197.34250943287</v>
+        <v>46197.50917609954</v>
       </c>
       <c r="D65" s="8">
-        <v>46197.34252800926</v>
+        <v>46197.50919467593</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>248</v>
@@ -5466,13 +5466,13 @@
         <v>251</v>
       </c>
       <c r="B66" s="5">
-        <v>46073.62818190972</v>
+        <v>46073.79484857639</v>
       </c>
       <c r="C66" s="5">
-        <v>46197.34251795139</v>
+        <v>46197.50918461806</v>
       </c>
       <c r="D66" s="5">
-        <v>46197.34253938658</v>
+        <v>46197.50920605324</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>252</v>
@@ -5531,13 +5531,13 @@
         <v>254</v>
       </c>
       <c r="B67" s="8">
-        <v>46073.628182175926</v>
+        <v>46073.79484884259</v>
       </c>
       <c r="C67" s="8">
-        <v>46197.3425265625</v>
+        <v>46197.50919322917</v>
       </c>
       <c r="D67" s="8">
-        <v>46197.342540694444</v>
+        <v>46197.509207361116</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>255</v>
@@ -5596,13 +5596,13 @@
         <v>257</v>
       </c>
       <c r="B68" s="5">
-        <v>46076.45626391204</v>
+        <v>46076.6229305787</v>
       </c>
       <c r="C68" s="5">
-        <v>46197.342535393516</v>
+        <v>46197.50920206019</v>
       </c>
       <c r="D68" s="5">
-        <v>46197.34255072917</v>
+        <v>46197.50921739583</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>258</v>
@@ -5661,13 +5661,13 @@
         <v>260</v>
       </c>
       <c r="B69" s="8">
-        <v>46073.6281824537</v>
+        <v>46073.79484912037</v>
       </c>
       <c r="C69" s="8">
-        <v>46197.34258650463</v>
+        <v>46197.5092531713</v>
       </c>
       <c r="D69" s="8">
-        <v>46197.34260322917</v>
+        <v>46197.50926989583</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>194</v>
@@ -5724,13 +5724,13 @@
         <v>263</v>
       </c>
       <c r="B70" s="5">
-        <v>46073.6281827662</v>
+        <v>46073.794849432874</v>
       </c>
       <c r="C70" s="5">
-        <v>46197.34263151621</v>
+        <v>46197.50929818287</v>
       </c>
       <c r="D70" s="5">
-        <v>46197.342655127315</v>
+        <v>46197.50932179399</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>195</v>
@@ -5787,11 +5787,11 @@
         <v>265</v>
       </c>
       <c r="B71" s="8">
-        <v>46073.6281803125</v>
+        <v>46073.794846979166</v>
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46090.50283079861</v>
+        <v>46090.66949746528</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>266</v>
@@ -5834,11 +5834,11 @@
         <v>268</v>
       </c>
       <c r="B72" s="5">
-        <v>46073.62818071759</v>
+        <v>46073.794847384255</v>
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46197.342650624996</v>
+        <v>46197.50931729167</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>269</v>
@@ -5895,11 +5895,11 @@
         <v>273</v>
       </c>
       <c r="B73" s="8">
-        <v>46073.62818100695</v>
+        <v>46073.79484767361</v>
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46179.00153725695</v>
+        <v>46179.16820392361</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>274</v>
@@ -5958,11 +5958,11 @@
         <v>277</v>
       </c>
       <c r="B74" s="5">
-        <v>46073.6281812963</v>
+        <v>46073.79484796296</v>
       </c>
       <c r="C74" s="6"/>
       <c r="D74" s="5">
-        <v>46182.01569325231</v>
+        <v>46182.18235991898</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>278</v>
@@ -6019,11 +6019,11 @@
         <v>280</v>
       </c>
       <c r="B75" s="8">
-        <v>46073.62818158565</v>
+        <v>46073.79484825231</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46183.02135520833</v>
+        <v>46183.188021875</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>281</v>
@@ -6080,11 +6080,11 @@
         <v>283</v>
       </c>
       <c r="B76" s="5">
-        <v>46073.628181886575</v>
+        <v>46073.79484855324</v>
       </c>
       <c r="C76" s="6"/>
       <c r="D76" s="5">
-        <v>46090.50286570602</v>
+        <v>46090.66953237269</v>
       </c>
       <c r="E76" s="6" t="s">
         <v>284</v>
@@ -6127,11 +6127,11 @@
         <v>286</v>
       </c>
       <c r="B77" s="8">
-        <v>46073.62818219907</v>
+        <v>46073.79484886574</v>
       </c>
       <c r="C77" s="9"/>
       <c r="D77" s="8">
-        <v>46192.00885878473</v>
+        <v>46192.175525451385</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>287</v>
@@ -6190,11 +6190,11 @@
         <v>291</v>
       </c>
       <c r="B78" s="5">
-        <v>46073.62818248842</v>
+        <v>46073.79484915509</v>
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46192.00885878473</v>
+        <v>46192.175525451385</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>292</v>
@@ -6253,11 +6253,11 @@
         <v>293</v>
       </c>
       <c r="B79" s="8">
-        <v>46090.47971854167</v>
+        <v>46090.64638520833</v>
       </c>
       <c r="C79" s="9"/>
       <c r="D79" s="8">
-        <v>46090.50289863426</v>
+        <v>46090.66956530092</v>
       </c>
       <c r="E79" s="9" t="s">
         <v>294</v>
@@ -6300,11 +6300,11 @@
         <v>296</v>
       </c>
       <c r="B80" s="5">
-        <v>46090.47982414352</v>
+        <v>46090.646490810184</v>
       </c>
       <c r="C80" s="6"/>
       <c r="D80" s="5">
-        <v>46191.020989675926</v>
+        <v>46191.18765634259</v>
       </c>
       <c r="E80" s="6" t="s">
         <v>297</v>
@@ -6363,11 +6363,11 @@
         <v>299</v>
       </c>
       <c r="B81" s="8">
-        <v>46090.48022813657</v>
+        <v>46090.64689480324</v>
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46192.00939141204</v>
+        <v>46192.17605807871</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>300</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-24 21:46 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="302">
   <si>
     <t>50001446-MINERA FRESNILLO</t>
   </si>
@@ -934,6 +934,10 @@
   </si>
   <si>
     <t>PACKING LIST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjunto PL.
+https://app.asana.com/1/402967058777498/profile/1213576320894219 quedo atento a tus comentarios si es necesario realizar una modificación o incluir más bultos</t>
   </si>
   <si>
     <t>Despacho,Logistica:</t>
@@ -5791,7 +5795,7 @@
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46090.66949746528</v>
+        <v>46197.90012883102</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>266</v>
@@ -5960,9 +5964,11 @@
       <c r="B74" s="5">
         <v>46073.79484796296</v>
       </c>
-      <c r="C74" s="6"/>
+      <c r="C74" s="5">
+        <v>46197.90011859954</v>
+      </c>
       <c r="D74" s="5">
-        <v>46182.18235991898</v>
+        <v>46197.90013689815</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>278</v>
@@ -5984,7 +5990,7 @@
         <v>26</v>
       </c>
       <c r="L74" s="6" t="s">
-        <v>26</v>
+        <v>279</v>
       </c>
       <c r="M74" s="6" t="s">
         <v>26</v>
@@ -5996,7 +6002,7 @@
         <v>274</v>
       </c>
       <c r="P74" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q74" s="5">
         <v>46181</v>
@@ -6008,25 +6014,25 @@
         <v>60</v>
       </c>
       <c r="T74" s="6">
-        <v>0</v>
-      </c>
-      <c r="U74" s="10" t="s">
-        <v>61</v>
+        <v>1</v>
+      </c>
+      <c r="U74" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A75" s="7" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B75" s="8">
         <v>46073.79484825231</v>
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46183.188021875</v>
+        <v>46197.90013631944</v>
       </c>
       <c r="E75" s="9" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="F75" s="9" t="s">
         <v>26</v>
@@ -6057,7 +6063,7 @@
         <v>278</v>
       </c>
       <c r="P75" s="9" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Q75" s="8">
         <v>46182</v>
@@ -6071,13 +6077,13 @@
       <c r="T75" s="9">
         <v>0</v>
       </c>
-      <c r="U75" s="10" t="s">
-        <v>61</v>
+      <c r="U75" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A76" s="4" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B76" s="5">
         <v>46073.79484855324</v>
@@ -6087,7 +6093,7 @@
         <v>46090.66953237269</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F76" s="6" t="s">
         <v>25</v>
@@ -6111,7 +6117,7 @@
         <v>26</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>26</v>
@@ -6124,7 +6130,7 @@
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A77" s="7" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B77" s="8">
         <v>46073.79484886574</v>
@@ -6134,16 +6140,16 @@
         <v>46192.175525451385</v>
       </c>
       <c r="E77" s="9" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="F77" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G77" s="9" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H77" s="9" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I77" s="8">
         <v>46182</v>
@@ -6161,13 +6167,13 @@
         <v>26</v>
       </c>
       <c r="N77" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="O77" s="9" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="P77" s="9" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q77" s="8">
         <v>46183</v>
@@ -6187,7 +6193,7 @@
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A78" s="4" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="B78" s="5">
         <v>46073.79484915509</v>
@@ -6197,16 +6203,16 @@
         <v>46192.175525451385</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="F78" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H78" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="I78" s="5">
         <v>46182</v>
@@ -6224,13 +6230,13 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P78" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Q78" s="5">
         <v>46183</v>
@@ -6250,7 +6256,7 @@
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B79" s="8">
         <v>46090.64638520833</v>
@@ -6260,7 +6266,7 @@
         <v>46090.66956530092</v>
       </c>
       <c r="E79" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="F79" s="9" t="s">
         <v>25</v>
@@ -6284,7 +6290,7 @@
         <v>26</v>
       </c>
       <c r="O79" s="9" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="P79" s="9" t="s">
         <v>26</v>
@@ -6297,7 +6303,7 @@
     </row>
     <row r="80" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A80" s="4" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B80" s="5">
         <v>46090.646490810184</v>
@@ -6307,7 +6313,7 @@
         <v>46191.18765634259</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F80" s="6" t="s">
         <v>26</v>
@@ -6334,13 +6340,13 @@
         <v>26</v>
       </c>
       <c r="N80" s="6" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="P80" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="Q80" s="5">
         <v>46182</v>
@@ -6360,7 +6366,7 @@
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A81" s="7" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B81" s="8">
         <v>46090.64689480324</v>
@@ -6370,7 +6376,7 @@
         <v>46192.17605807871</v>
       </c>
       <c r="E81" s="9" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="F81" s="9" t="s">
         <v>26</v>
@@ -6397,13 +6403,13 @@
         <v>26</v>
       </c>
       <c r="N81" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="O81" s="9" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="P81" s="9" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Q81" s="8">
         <v>46191</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-25 13:19 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -4181,9 +4181,11 @@
       <c r="B45" s="8">
         <v>46073.794849467595</v>
       </c>
-      <c r="C45" s="9"/>
+      <c r="C45" s="8">
+        <v>46198.551042673615</v>
+      </c>
       <c r="D45" s="8">
-        <v>46114.798811886576</v>
+        <v>46198.55105587963</v>
       </c>
       <c r="E45" s="9" t="s">
         <v>174</v>
@@ -4218,9 +4220,11 @@
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
       <c r="S45" s="9"/>
-      <c r="T45" s="9"/>
-      <c r="U45" s="12" t="s">
-        <v>81</v>
+      <c r="T45" s="9">
+        <v>1</v>
+      </c>
+      <c r="U45" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
@@ -4423,9 +4427,11 @@
       <c r="B49" s="8">
         <v>46087.810021701385</v>
       </c>
-      <c r="C49" s="9"/>
+      <c r="C49" s="8">
+        <v>46198.55102407407</v>
+      </c>
       <c r="D49" s="8">
-        <v>46197.50927037037</v>
+        <v>46198.551042928244</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>191</v>
@@ -4471,10 +4477,10 @@
         <v>60</v>
       </c>
       <c r="T49" s="9">
-        <v>0</v>
-      </c>
-      <c r="U49" s="12" t="s">
-        <v>81</v>
+        <v>1</v>
+      </c>
+      <c r="U49" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
@@ -5734,7 +5740,7 @@
         <v>46197.50929818287</v>
       </c>
       <c r="D70" s="5">
-        <v>46197.50932179399</v>
+        <v>46198.55104168982</v>
       </c>
       <c r="E70" s="6" t="s">
         <v>195</v>
@@ -5782,8 +5788,8 @@
       <c r="T70" s="6">
         <v>1</v>
       </c>
-      <c r="U70" s="11" t="s">
-        <v>33</v>
+      <c r="U70" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="71" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-27 19:35 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -6379,7 +6379,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46199.25036193287</v>
+        <v>46200.17552224537</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>301</v>
@@ -6429,8 +6429,8 @@
       <c r="T81" s="9">
         <v>0</v>
       </c>
-      <c r="U81" s="12" t="s">
-        <v>81</v>
+      <c r="U81" s="10" t="s">
+        <v>61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-07-01 18:30 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -909,10 +909,10 @@
     <t>Coordinacion Entrega con Cliente</t>
   </si>
   <si>
-    <t>Francisca Alejandra Ramos Aravales</t>
-  </si>
-  <si>
-    <t>francisca@zitron.com</t>
+    <t>Karin Pinto</t>
+  </si>
+  <si>
+    <t>kpinto@zitron.com</t>
   </si>
   <si>
     <t>Embalaje,Logistica:</t>
@@ -5848,7 +5848,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46197.50931729167</v>
+        <v>46204.69436715278</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>269</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-07 13:36 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -5909,7 +5909,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46179.16820392361</v>
+        <v>46209.925254525464</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>274</v>
@@ -5957,10 +5957,10 @@
         <v>60</v>
       </c>
       <c r="T73" s="9">
-        <v>0</v>
-      </c>
-      <c r="U73" s="10" t="s">
-        <v>61</v>
+        <v>0.7</v>
+      </c>
+      <c r="U73" s="12" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-12 19:40 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -213,12 +213,6 @@
   </si>
   <si>
     <t>Embalaje,Ingenieria Servicios:</t>
-  </si>
-  <si>
-    <t>Baja</t>
-  </si>
-  <si>
-    <t>Tarea sin iniciar</t>
   </si>
   <si>
     <t>1213330955220903</t>
@@ -447,6 +441,9 @@
     <t>Generación OC Alabe,Fabricación Alabe</t>
   </si>
   <si>
+    <t>Baja</t>
+  </si>
+  <si>
     <t>1213330955220917</t>
   </si>
   <si>
@@ -454,6 +451,9 @@
   </si>
   <si>
     <t>Fabricación Alabe,Alabe</t>
+  </si>
+  <si>
+    <t>Tarea sin iniciar</t>
   </si>
   <si>
     <t>1213330955220918</t>
@@ -2097,7 +2097,7 @@
         <v>46129.60127643518</v>
       </c>
       <c r="D12" s="5">
-        <v>46154.171658692125</v>
+        <v>46246.80198226852</v>
       </c>
       <c r="E12" s="6" t="s">
         <v>57</v>
@@ -2141,19 +2141,19 @@
       <c r="R12" s="5">
         <v>46153</v>
       </c>
-      <c r="S12" s="11" t="s">
-        <v>60</v>
+      <c r="S12" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T12" s="6">
         <v>1</v>
       </c>
-      <c r="U12" s="10" t="s">
-        <v>61</v>
+      <c r="U12" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B13" s="8">
         <v>46073.794849513884</v>
@@ -2165,7 +2165,7 @@
         <v>46129.71444074074</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>25</v>
@@ -2189,7 +2189,7 @@
         <v>26</v>
       </c>
       <c r="O13" s="9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="P13" s="9" t="s">
         <v>26</v>
@@ -2202,7 +2202,7 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46073.79484703703</v>
@@ -2214,7 +2214,7 @@
         <v>46104.554936064815</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>26</v>
@@ -2235,19 +2235,19 @@
         <v>26</v>
       </c>
       <c r="L14" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="M14" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N14" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O14" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P14" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="Q14" s="5">
         <v>46014</v>
@@ -2267,7 +2267,7 @@
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B15" s="8">
         <v>46073.794847592595</v>
@@ -2279,7 +2279,7 @@
         <v>46104.55553096065</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F15" s="9" t="s">
         <v>26</v>
@@ -2300,19 +2300,19 @@
         <v>26</v>
       </c>
       <c r="L15" s="9" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="M15" s="9" t="s">
         <v>26</v>
       </c>
       <c r="N15" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O15" s="9" t="s">
         <v>42</v>
       </c>
       <c r="P15" s="9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="Q15" s="8">
         <v>46014</v>
@@ -2332,7 +2332,7 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B16" s="5">
         <v>46073.79484783565</v>
@@ -2344,7 +2344,7 @@
         <v>46104.56897644676</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F16" s="6" t="s">
         <v>26</v>
@@ -2365,19 +2365,19 @@
         <v>26</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O16" s="6" t="s">
         <v>42</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="Q16" s="5">
         <v>46014</v>
@@ -2397,7 +2397,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B17" s="8">
         <v>46073.79484809028</v>
@@ -2409,7 +2409,7 @@
         <v>46100.77890356482</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F17" s="9" t="s">
         <v>26</v>
@@ -2436,13 +2436,13 @@
         <v>26</v>
       </c>
       <c r="N17" s="9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="O17" s="9" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="P17" s="9" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="Q17" s="8">
         <v>46014</v>
@@ -2457,12 +2457,12 @@
         <v>1</v>
       </c>
       <c r="U17" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B18" s="5">
         <v>46073.79484833333</v>
@@ -2474,7 +2474,7 @@
         <v>46114.50370078704</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F18" s="6" t="s">
         <v>25</v>
@@ -2498,7 +2498,7 @@
         <v>26</v>
       </c>
       <c r="O18" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="P18" s="6" t="s">
         <v>26</v>
@@ -2515,7 +2515,7 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B19" s="8">
         <v>46073.79484857639</v>
@@ -2527,7 +2527,7 @@
         <v>46104.56950603009</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>26</v>
@@ -2548,19 +2548,19 @@
         <v>26</v>
       </c>
       <c r="L19" s="9" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="M19" s="9" t="s">
         <v>26</v>
       </c>
       <c r="N19" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="O19" s="9" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P19" s="9" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="Q19" s="8">
         <v>46023</v>
@@ -2580,7 +2580,7 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B20" s="5">
         <v>46073.79484880787</v>
@@ -2592,7 +2592,7 @@
         <v>46104.56972186343</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F20" s="6" t="s">
         <v>26</v>
@@ -2613,19 +2613,19 @@
         <v>26</v>
       </c>
       <c r="L20" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="M20" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="Q20" s="5">
         <v>46016</v>
@@ -2645,7 +2645,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B21" s="8">
         <v>46073.79484905093</v>
@@ -2657,7 +2657,7 @@
         <v>46104.570394375</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>26</v>
@@ -2678,19 +2678,19 @@
         <v>26</v>
       </c>
       <c r="L21" s="9" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="M21" s="9" t="s">
         <v>26</v>
       </c>
       <c r="N21" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="O21" s="9" t="s">
         <v>52</v>
       </c>
       <c r="P21" s="9" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="Q21" s="8">
         <v>46017</v>
@@ -2710,7 +2710,7 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B22" s="5">
         <v>46073.79484929398</v>
@@ -2722,16 +2722,16 @@
         <v>46223.80841302083</v>
       </c>
       <c r="E22" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G22" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="I22" s="5">
         <v>46023</v>
@@ -2749,13 +2749,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="Q22" s="5">
         <v>46023</v>
@@ -2775,7 +2775,7 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B23" s="8">
         <v>46076.58214225694</v>
@@ -2787,7 +2787,7 @@
         <v>46114.503793055555</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F23" s="9" t="s">
         <v>26</v>
@@ -2814,13 +2814,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="9" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="O23" s="9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P23" s="9" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="Q23" s="8">
         <v>46023</v>
@@ -2840,7 +2840,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B24" s="5">
         <v>46073.79484642361</v>
@@ -2852,16 +2852,16 @@
         <v>46223.80840997685</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I24" s="5">
         <v>46023</v>
@@ -2879,13 +2879,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="Q24" s="5">
         <v>46023</v>
@@ -2905,7 +2905,7 @@
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B25" s="8">
         <v>46073.79484674768</v>
@@ -2917,7 +2917,7 @@
         <v>46129.71472099537</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F25" s="9" t="s">
         <v>25</v>
@@ -2941,7 +2941,7 @@
         <v>26</v>
       </c>
       <c r="O25" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="P25" s="9" t="s">
         <v>26</v>
@@ -2958,7 +2958,7 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B26" s="5">
         <v>46073.79484700231</v>
@@ -2970,16 +2970,16 @@
         <v>46134.20558688657</v>
       </c>
       <c r="E26" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>112</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G26" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>114</v>
       </c>
       <c r="I26" s="5">
         <v>46027</v>
@@ -2997,13 +2997,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q26" s="5">
         <v>46027</v>
@@ -3012,18 +3012,18 @@
         <v>46141</v>
       </c>
       <c r="S26" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T26" s="6">
         <v>1</v>
       </c>
       <c r="U26" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B27" s="8">
         <v>46073.794847268524</v>
@@ -3035,16 +3035,16 @@
         <v>46101.813124513894</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I27" s="8">
         <v>46027</v>
@@ -3062,13 +3062,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="O27" s="9" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="Q27" s="8">
         <v>46027</v>
@@ -3077,13 +3077,13 @@
         <v>46028</v>
       </c>
       <c r="S27" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T27" s="9">
         <v>0</v>
       </c>
       <c r="U27" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
@@ -3106,10 +3106,10 @@
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I28" s="5">
         <v>46029</v>
@@ -3127,10 +3127,10 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="P28" s="6" t="s">
         <v>121</v>
@@ -3142,13 +3142,13 @@
         <v>46141</v>
       </c>
       <c r="S28" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T28" s="6">
         <v>0</v>
       </c>
       <c r="U28" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
@@ -3171,10 +3171,10 @@
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I29" s="8">
         <v>46027</v>
@@ -3192,13 +3192,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O29" s="9" t="s">
         <v>124</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q29" s="8">
         <v>46027</v>
@@ -3207,13 +3207,13 @@
         <v>46141</v>
       </c>
       <c r="S29" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T29" s="9">
         <v>1</v>
       </c>
       <c r="U29" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
@@ -3236,10 +3236,10 @@
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I30" s="5">
         <v>46027</v>
@@ -3260,7 +3260,7 @@
         <v>123</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>127</v>
@@ -3268,13 +3268,13 @@
       <c r="Q30" s="6"/>
       <c r="R30" s="6"/>
       <c r="S30" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T30" s="6">
         <v>0</v>
       </c>
       <c r="U30" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
@@ -3297,10 +3297,10 @@
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I31" s="8">
         <v>46036</v>
@@ -3329,13 +3329,13 @@
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
       <c r="S31" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T31" s="9">
         <v>0</v>
       </c>
       <c r="U31" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -3358,10 +3358,10 @@
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I32" s="5">
         <v>46027</v>
@@ -3379,13 +3379,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O32" s="6" t="s">
         <v>133</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q32" s="5">
         <v>46027</v>
@@ -3423,10 +3423,10 @@
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I33" s="8">
         <v>46027</v>
@@ -3447,7 +3447,7 @@
         <v>132</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="P33" s="9" t="s">
         <v>136</v>
@@ -3455,13 +3455,13 @@
       <c r="Q33" s="9"/>
       <c r="R33" s="9"/>
       <c r="S33" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T33" s="9">
         <v>0</v>
       </c>
       <c r="U33" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
@@ -3484,10 +3484,10 @@
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I34" s="5">
         <v>46029</v>
@@ -3516,13 +3516,13 @@
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
       <c r="S34" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T34" s="6">
         <v>0</v>
       </c>
       <c r="U34" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
@@ -3545,10 +3545,10 @@
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I35" s="8">
         <v>46020</v>
@@ -3566,13 +3566,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O35" s="9" t="s">
         <v>142</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q35" s="8">
         <v>46020</v>
@@ -3581,13 +3581,13 @@
         <v>46164</v>
       </c>
       <c r="S35" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T35" s="9">
         <v>1</v>
       </c>
       <c r="U35" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
@@ -3610,10 +3610,10 @@
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I36" s="5">
         <v>46020</v>
@@ -3634,7 +3634,7 @@
         <v>141</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>145</v>
@@ -3642,13 +3642,13 @@
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
       <c r="S36" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T36" s="6">
         <v>0</v>
       </c>
       <c r="U36" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
@@ -3671,10 +3671,10 @@
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I37" s="8">
         <v>46038</v>
@@ -3703,13 +3703,13 @@
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
       <c r="S37" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T37" s="9">
         <v>0</v>
       </c>
       <c r="U37" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
@@ -3732,10 +3732,10 @@
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I38" s="5">
         <v>46038</v>
@@ -3764,13 +3764,13 @@
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
       <c r="S38" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T38" s="6">
         <v>0</v>
       </c>
       <c r="U38" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
@@ -3814,13 +3814,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O39" s="9" t="s">
         <v>156</v>
       </c>
       <c r="P39" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q39" s="8">
         <v>46024</v>
@@ -3882,7 +3882,7 @@
         <v>153</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="P40" s="6" t="s">
         <v>159</v>
@@ -3890,13 +3890,13 @@
       <c r="Q40" s="6"/>
       <c r="R40" s="6"/>
       <c r="S40" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T40" s="6">
         <v>0</v>
       </c>
       <c r="U40" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
@@ -3951,13 +3951,13 @@
       <c r="Q41" s="9"/>
       <c r="R41" s="9"/>
       <c r="S41" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T41" s="9">
         <v>0</v>
       </c>
       <c r="U41" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
@@ -4001,13 +4001,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="O42" s="6" t="s">
         <v>165</v>
       </c>
       <c r="P42" s="6" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="Q42" s="5">
         <v>46027</v>
@@ -4016,13 +4016,13 @@
         <v>46133</v>
       </c>
       <c r="S42" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T42" s="6">
         <v>1</v>
       </c>
       <c r="U42" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
@@ -4069,7 +4069,7 @@
         <v>164</v>
       </c>
       <c r="O43" s="9" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="P43" s="9" t="s">
         <v>168</v>
@@ -4077,13 +4077,13 @@
       <c r="Q43" s="9"/>
       <c r="R43" s="9"/>
       <c r="S43" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T43" s="9">
         <v>0</v>
       </c>
       <c r="U43" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
@@ -4138,13 +4138,13 @@
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
       <c r="S44" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T44" s="6">
         <v>0</v>
       </c>
       <c r="U44" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
@@ -4244,7 +4244,7 @@
         <v>173</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="P46" s="6" t="s">
         <v>179</v>
@@ -4447,7 +4447,7 @@
         <v>46171</v>
       </c>
       <c r="S49" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T49" s="9">
         <v>1</v>
@@ -4565,7 +4565,7 @@
         <v>46076</v>
       </c>
       <c r="S51" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T51" s="9">
         <v>1</v>
@@ -4630,7 +4630,7 @@
         <v>46078</v>
       </c>
       <c r="S52" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T52" s="6">
         <v>1</v>
@@ -4748,7 +4748,7 @@
         <v>46087</v>
       </c>
       <c r="S54" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T54" s="6">
         <v>1</v>
@@ -4813,7 +4813,7 @@
         <v>46118</v>
       </c>
       <c r="S55" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T55" s="9">
         <v>1</v>
@@ -4878,7 +4878,7 @@
         <v>46120</v>
       </c>
       <c r="S56" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T56" s="6">
         <v>1</v>
@@ -5057,13 +5057,13 @@
         <v>46146</v>
       </c>
       <c r="S59" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T59" s="9">
         <v>1</v>
       </c>
       <c r="U59" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -5122,13 +5122,13 @@
         <v>46146</v>
       </c>
       <c r="S60" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T60" s="6">
         <v>1</v>
       </c>
       <c r="U60" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5187,13 +5187,13 @@
         <v>46168</v>
       </c>
       <c r="S61" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T61" s="9">
         <v>1</v>
       </c>
       <c r="U61" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5252,13 +5252,13 @@
         <v>46135</v>
       </c>
       <c r="S62" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T62" s="6">
         <v>1</v>
       </c>
       <c r="U62" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5334,10 +5334,10 @@
         <v>26</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H64" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I64" s="5">
         <v>46121</v>
@@ -5370,7 +5370,7 @@
         <v>46129</v>
       </c>
       <c r="S64" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T64" s="6">
         <v>1</v>
@@ -5399,10 +5399,10 @@
         <v>26</v>
       </c>
       <c r="G65" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H65" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I65" s="8">
         <v>46168</v>
@@ -5435,7 +5435,7 @@
         <v>46170</v>
       </c>
       <c r="S65" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T65" s="9">
         <v>1</v>
@@ -5464,10 +5464,10 @@
         <v>26</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H66" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I66" s="5">
         <v>46147</v>
@@ -5500,7 +5500,7 @@
         <v>46148</v>
       </c>
       <c r="S66" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T66" s="6">
         <v>1</v>
@@ -5529,10 +5529,10 @@
         <v>26</v>
       </c>
       <c r="G67" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H67" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I67" s="8">
         <v>46149</v>
@@ -5565,7 +5565,7 @@
         <v>46120</v>
       </c>
       <c r="S67" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T67" s="9">
         <v>1</v>
@@ -5594,10 +5594,10 @@
         <v>26</v>
       </c>
       <c r="G68" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H68" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I68" s="5">
         <v>46136</v>
@@ -5630,7 +5630,7 @@
         <v>46140</v>
       </c>
       <c r="S68" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T68" s="6">
         <v>1</v>
@@ -5659,10 +5659,10 @@
         <v>26</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H69" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I69" s="9"/>
       <c r="J69" s="8">
@@ -5693,7 +5693,7 @@
         <v>46170</v>
       </c>
       <c r="S69" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T69" s="9">
         <v>1</v>
@@ -5722,10 +5722,10 @@
         <v>26</v>
       </c>
       <c r="G70" s="6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H70" s="6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I70" s="6"/>
       <c r="J70" s="5">
@@ -5756,7 +5756,7 @@
         <v>46172</v>
       </c>
       <c r="S70" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T70" s="6">
         <v>1</v>
@@ -5821,7 +5821,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46211.69907109954</v>
+        <v>46246.80485579861</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>268</v>
@@ -5863,14 +5863,14 @@
       <c r="R72" s="5">
         <v>46175</v>
       </c>
-      <c r="S72" s="11" t="s">
-        <v>60</v>
+      <c r="S72" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T72" s="6">
         <v>0</v>
       </c>
       <c r="U72" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="73" spans="1:21" x14ac:dyDescent="0.25">
@@ -5882,7 +5882,7 @@
       </c>
       <c r="C73" s="9"/>
       <c r="D73" s="8">
-        <v>46223.83377060185</v>
+        <v>46246.80485609954</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>273</v>
@@ -5891,10 +5891,10 @@
         <v>26</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H73" s="9" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="I73" s="8">
         <v>46175</v>
@@ -5926,14 +5926,14 @@
       <c r="R73" s="8">
         <v>46178</v>
       </c>
-      <c r="S73" s="11" t="s">
-        <v>60</v>
+      <c r="S73" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T73" s="9">
         <v>0.7</v>
       </c>
       <c r="U73" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5947,7 +5947,7 @@
         <v>46197.90011859954</v>
       </c>
       <c r="D74" s="5">
-        <v>46241.909162951386</v>
+        <v>46246.804856400464</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>277</v>
@@ -5989,8 +5989,8 @@
       <c r="R74" s="5">
         <v>46181</v>
       </c>
-      <c r="S74" s="11" t="s">
-        <v>60</v>
+      <c r="S74" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T74" s="6">
         <v>1</v>
@@ -6008,7 +6008,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46240.72403283565</v>
+        <v>46246.80485667824</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>281</v>
@@ -6050,14 +6050,14 @@
       <c r="R75" s="8">
         <v>46182</v>
       </c>
-      <c r="S75" s="11" t="s">
-        <v>60</v>
+      <c r="S75" s="10" t="s">
+        <v>32</v>
       </c>
       <c r="T75" s="9">
         <v>0</v>
       </c>
       <c r="U75" s="12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">
@@ -6161,13 +6161,13 @@
         <v>46191</v>
       </c>
       <c r="S77" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T77" s="9">
         <v>0</v>
       </c>
       <c r="U77" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6224,13 +6224,13 @@
         <v>46191</v>
       </c>
       <c r="S78" s="11" t="s">
-        <v>60</v>
+        <v>114</v>
       </c>
       <c r="T78" s="6">
         <v>0</v>
       </c>
       <c r="U78" s="10" t="s">
-        <v>61</v>
+        <v>118</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
KPI actualizado 2026-08-26 14:46 UTC
</commit_message>
<xml_diff>
--- a/data/50001446 - MINERA FRESNILLO.xlsx
+++ b/data/50001446 - MINERA FRESNILLO.xlsx
@@ -5774,7 +5774,7 @@
       </c>
       <c r="C71" s="9"/>
       <c r="D71" s="8">
-        <v>46197.90012883102</v>
+        <v>46260.59887969907</v>
       </c>
       <c r="E71" s="9" t="s">
         <v>265</v>
@@ -5880,9 +5880,11 @@
       <c r="B73" s="8">
         <v>46073.79484767361</v>
       </c>
-      <c r="C73" s="9"/>
+      <c r="C73" s="8">
+        <v>46260.59887023148</v>
+      </c>
       <c r="D73" s="8">
-        <v>46246.80485609954</v>
+        <v>46260.59888653935</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>273</v>
@@ -5930,10 +5932,10 @@
         <v>32</v>
       </c>
       <c r="T73" s="9">
-        <v>0.7</v>
-      </c>
-      <c r="U73" s="12" t="s">
-        <v>79</v>
+        <v>1</v>
+      </c>
+      <c r="U73" s="11" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="74" spans="1:21" x14ac:dyDescent="0.25">
@@ -5947,7 +5949,7 @@
         <v>46197.90011859954</v>
       </c>
       <c r="D74" s="5">
-        <v>46246.804856400464</v>
+        <v>46260.598887314816</v>
       </c>
       <c r="E74" s="6" t="s">
         <v>277</v>
@@ -5995,8 +5997,8 @@
       <c r="T74" s="6">
         <v>1</v>
       </c>
-      <c r="U74" s="11" t="s">
-        <v>33</v>
+      <c r="U74" s="12" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="75" spans="1:21" x14ac:dyDescent="0.25">
@@ -6008,7 +6010,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46246.80485667824</v>
+        <v>46260.594010381945</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>281</v>
@@ -6056,8 +6058,8 @@
       <c r="T75" s="9">
         <v>0</v>
       </c>
-      <c r="U75" s="12" t="s">
-        <v>79</v>
+      <c r="U75" s="10" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="76" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>